<commit_message>
Finalize project documentation and frontend cleanup
</commit_message>
<xml_diff>
--- a/project-management/bug-reports/Bug-Tracking.xlsx
+++ b/project-management/bug-reports/Bug-Tracking.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="69">
   <si>
     <t>Bug ID</t>
   </si>
@@ -29,15 +29,9 @@
     <t>Modül</t>
   </si>
   <si>
-    <t xml:space="preserve"> Hata Türü</t>
-  </si>
-  <si>
     <t>Açıklama</t>
   </si>
   <si>
-    <t>Severety</t>
-  </si>
-  <si>
     <t>Priority</t>
   </si>
   <si>
@@ -95,15 +89,9 @@
     <t>TC-04-01</t>
   </si>
   <si>
-    <t>Recommendation</t>
-  </si>
-  <si>
     <t>Age group filtering not applied</t>
   </si>
   <si>
-    <t>Test planning phase</t>
-  </si>
-  <si>
     <t>BR-02</t>
   </si>
   <si>
@@ -116,22 +104,124 @@
     <t>TC-05-02</t>
   </si>
   <si>
-    <t>Login</t>
-  </si>
-  <si>
     <t>Activity List</t>
   </si>
   <si>
     <t>Invalid credentials not handled clearly</t>
   </si>
   <si>
-    <t>UI validation case</t>
-  </si>
-  <si>
     <t>Empty result message not informative</t>
   </si>
   <si>
     <t>UX improvement</t>
+  </si>
+  <si>
+    <t>BR-04</t>
+  </si>
+  <si>
+    <t>TC-03-02</t>
+  </si>
+  <si>
+    <t>School Management</t>
+  </si>
+  <si>
+    <t>School update changes not saved to database</t>
+  </si>
+  <si>
+    <t>Resolved</t>
+  </si>
+  <si>
+    <t>Missing database commit fixed</t>
+  </si>
+  <si>
+    <t>BR-05</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Expired JWT token not handled correctly</t>
+  </si>
+  <si>
+    <t>Added centralized 401 handling</t>
+  </si>
+  <si>
+    <t>BR-06</t>
+  </si>
+  <si>
+    <t>TC-04-03</t>
+  </si>
+  <si>
+    <t>Configuration</t>
+  </si>
+  <si>
+    <t>BR-07</t>
+  </si>
+  <si>
+    <t>TC-05-04</t>
+  </si>
+  <si>
+    <t>BR-08</t>
+  </si>
+  <si>
+    <t>TC-06-02</t>
+  </si>
+  <si>
+    <t>AI Adaptation</t>
+  </si>
+  <si>
+    <t>Adapted activity difficult to identify after save</t>
+  </si>
+  <si>
+    <t>Activity traceability improved</t>
+  </si>
+  <si>
+    <t>BR-09</t>
+  </si>
+  <si>
+    <t>TC-07-01</t>
+  </si>
+  <si>
+    <t>Mobile Integration</t>
+  </si>
+  <si>
+    <t>Android app could not connect to local backend</t>
+  </si>
+  <si>
+    <t>Capacitor network configuration updated</t>
+  </si>
+  <si>
+    <t>Hata Türü</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Recommendation Engine</t>
+  </si>
+  <si>
+    <t>Recommendation filtering fixed</t>
+  </si>
+  <si>
+    <t>Authentication flow improved</t>
+  </si>
+  <si>
+    <t>Gemini Integration</t>
+  </si>
+  <si>
+    <t>Gemini dependency installation failed in CI pipeline</t>
+  </si>
+  <si>
+    <t>CI dependency configuration corrected</t>
+  </si>
+  <si>
+    <t>Activity Management</t>
+  </si>
+  <si>
+    <t>Activity planning fields not preserved during update</t>
+  </si>
+  <si>
+    <t>Extended planning field support added</t>
   </si>
 </sst>
 </file>
@@ -152,7 +242,6 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -164,7 +253,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -187,22 +276,432 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="16">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -213,6 +712,27 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Таблица1" displayName="Таблица1" ref="A1:L10" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="14" tableBorderDxfId="15" totalsRowBorderDxfId="13">
+  <autoFilter ref="A1:L10"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Bug ID" dataDxfId="12"/>
+    <tableColumn id="2" name="Sprint" dataDxfId="11"/>
+    <tableColumn id="3" name="Test Case ID" dataDxfId="10"/>
+    <tableColumn id="4" name="Modül" dataDxfId="9"/>
+    <tableColumn id="5" name="Hata Türü" dataDxfId="8"/>
+    <tableColumn id="6" name="Açıklama" dataDxfId="7"/>
+    <tableColumn id="7" name="Severity" dataDxfId="6"/>
+    <tableColumn id="8" name="Priority" dataDxfId="5"/>
+    <tableColumn id="9" name="Durum" dataDxfId="4"/>
+    <tableColumn id="10" name="Tespit Tarihi" dataDxfId="3"/>
+    <tableColumn id="11" name="Çözüm Tarihi" dataDxfId="2"/>
+    <tableColumn id="12" name="Notlar" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,169 +1022,409 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="6.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="42.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14" style="1" customWidth="1"/>
+    <col min="11" max="11" width="14.5703125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="43.42578125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>24</v>
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="B2" s="2">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="J2" s="3">
-        <v>46047</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>28</v>
+        <v>46162</v>
+      </c>
+      <c r="K2" s="3">
+        <v>46163</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>29</v>
+      <c r="A3" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="B3" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
-        <v>35</v>
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="J3" s="3">
-        <v>46047</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>36</v>
+        <v>46184</v>
+      </c>
+      <c r="K3" s="3">
+        <v>46185</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>30</v>
+      <c r="A4" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="3">
+        <v>46159</v>
+      </c>
+      <c r="K4" s="3">
+        <v>46159</v>
+      </c>
+      <c r="L4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="D5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="J5" s="3">
+        <v>46055</v>
+      </c>
+      <c r="K5" s="3">
+        <v>46056</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="2">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="3">
-        <v>46047</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>38</v>
+      <c r="I6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="3">
+        <v>46184</v>
+      </c>
+      <c r="K6" s="3">
+        <v>46185</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="2">
+        <v>6</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J7" s="3">
+        <v>46167</v>
+      </c>
+      <c r="K7" s="3">
+        <v>46168</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" s="3">
+        <v>46169</v>
+      </c>
+      <c r="K8" s="3">
+        <v>46169</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="2">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" s="3">
+        <v>46165</v>
+      </c>
+      <c r="K9" s="3">
+        <v>46166</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="10">
+        <v>8</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="J10" s="11">
+        <v>46108</v>
+      </c>
+      <c r="K10" s="11">
+        <v>46110</v>
+      </c>
+      <c r="L10" s="12" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -672,19 +1432,19 @@
           <x14:formula1>
             <xm:f>Лист1!$A$1:$A$5</xm:f>
           </x14:formula1>
-          <xm:sqref>E1:E1048576</xm:sqref>
+          <xm:sqref>E11:E1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Лист1!$C$1:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>G1:H1048576</xm:sqref>
+          <xm:sqref>G11:H1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Лист1!$E$1:$E$4</xm:f>
           </x14:formula1>
-          <xm:sqref>I1:I1048576</xm:sqref>
+          <xm:sqref>I11:I1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -699,48 +1459,48 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>